<commit_message>
Update environment ignore rules and blog tracker
</commit_message>
<xml_diff>
--- a/manual-files/wordpress-blog-content-tracker.xlsx
+++ b/manual-files/wordpress-blog-content-tracker.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B3713B7-607F-47A2-9A73-544E98F7C057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Blog tracker" state="visible" r:id="rId4"/>
+    <sheet name="Blog tracker" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
   <si>
     <t>blog_id</t>
   </si>
@@ -41,27 +42,30 @@
   </si>
   <si>
     <t>all of the files in a cuastom classic wordpress theme and how it works</t>
+  </si>
+  <si>
+    <t>pending</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="mmm dd, yyyy h:mm:ss AM/PM"/>
+    <numFmt numFmtId="164" formatCode="mmm\ dd\,\ yyyy\ h:mm:ss\ AM/PM"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -445,9 +449,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="42" customWidth="1"/>
@@ -455,7 +459,7 @@
     <col min="4" max="5" width="29" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -472,7 +476,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -483,10 +487,10 @@
         <v>6</v>
       </c>
       <c r="D2" s="1">
-        <v>46225.67197309028</v>
+        <v>46225.671973090277</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -500,7 +504,7 @@
         <v>46225.672587685185</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -508,23 +512,20 @@
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D4" s="1">
-        <v>46225.67486560185</v>
+        <v>46225.674865601854</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E1"/>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="C10:C200">
-      <formula1>"pending,complete,uploaded"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C2:C200">
+  <autoFilter ref="A1:E1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="C2:C200" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"pending,complete,uploaded"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>